<commit_message>
Update Astral Radiance progress and resources
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Astral_Radiance_Tracker.xlsx
+++ b/Astral_Radiance_Tracker.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="55">
   <si>
     <t xml:space="preserve">Astral Radiance Milestone Tracker</t>
   </si>
@@ -86,18 +86,21 @@
     <t xml:space="preserve">100 shards each of Doctor Strange, Ancient One, Moondragon and Emma Frost (X-Men)</t>
   </si>
   <si>
+    <t xml:space="preserve">Claimed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doctor Strange to 7 red stars + 150,000 gold + 15 training materials + 1,200 blue tokens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moondragon to 7 red stars + 150,000 gold + 20 training materials + 1,500 blue tokens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ancient One to 7 red stars + 200,000 gold + 25 training materials + 1,600 blue tokens</t>
+  </si>
+  <si>
     <t xml:space="preserve">Not claimed</t>
   </si>
   <si>
-    <t xml:space="preserve">Doctor Strange to 7 red stars + 150,000 gold + 15 training materials + 1,200 blue tokens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Moondragon to 7 red stars + 150,000 gold + 20 training materials + 1,500 blue tokens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ancient One to 7 red stars + 200,000 gold + 25 training materials + 1,600 blue tokens</t>
-  </si>
-  <si>
     <t xml:space="preserve">Emma Frost (X-Men) to 7 red stars + 250,000 gold + 30 training materials + 1,800 blue tokens</t>
   </si>
   <si>
@@ -111,6 +114,12 @@
   </si>
   <si>
     <t xml:space="preserve">Not in screenshots yet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diamond 5 character + 400,000 gold + 100 training materials + 4,600 blue tokens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final milestone. Out of reach with the listed tasks</t>
   </si>
   <si>
     <t xml:space="preserve">How to earn points</t>
@@ -704,14 +713,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>28750</v>
+        <v>34750</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">B6+Scoring!F12</f>
-        <v>70750</v>
+        <v>76750</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -720,7 +729,7 @@
       </c>
       <c r="B7" s="3" t="n">
         <f aca="false">SUMPRODUCT((B13:B25&lt;&gt;"")*(B13:B25&lt;=B6))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>8</v>
@@ -736,14 +745,14 @@
       </c>
       <c r="B8" s="3" t="n">
         <f aca="false">IFERROR(INDEX(A13:A25,MATCH(TRUE(),INDEX(B13:B25&gt;B6,0),0)),"All done")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E8" s="3" t="n">
         <f aca="false">SUMPRODUCT((B13:B25&lt;&gt;"")*(B13:B25&lt;=B6)*(F13:F25&lt;&gt;"Claimed"))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -752,7 +761,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IFERROR(INDEX(E13:E25,MATCH(TRUE(),INDEX(B13:B25&gt;B6,0),0)),0)</f>
-        <v>1250</v>
+        <v>5250</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -761,7 +770,7 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">MAX(0,MAX(B13:B25)-B6)</f>
-        <v>41250</v>
+        <v>165250</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -770,7 +779,7 @@
       </c>
       <c r="B11" s="6" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>6557.15357017808</v>
+        <v>27046.3804123115</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -844,7 +853,7 @@
       <c r="D15" s="10"/>
       <c r="E15" s="11" t="n">
         <f aca="false">IF(B15="","",MAX(0,B15-$B$6))</f>
-        <v>1250</v>
+        <v>0</v>
       </c>
       <c r="F15" s="12" t="s">
         <v>21</v>
@@ -863,10 +872,10 @@
       <c r="D16" s="10"/>
       <c r="E16" s="11" t="n">
         <f aca="false">IF(B16="","",MAX(0,B16-$B$6))</f>
-        <v>11250</v>
+        <v>5250</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -877,15 +886,15 @@
         <v>50000</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="11" t="n">
         <f aca="false">IF(B17="","",MAX(0,B17-$B$6))</f>
-        <v>21250</v>
+        <v>15250</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -896,15 +905,15 @@
         <v>60000</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D18" s="10"/>
       <c r="E18" s="11" t="n">
         <f aca="false">IF(B18="","",MAX(0,B18-$B$6))</f>
-        <v>31250</v>
+        <v>25250</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -915,17 +924,17 @@
         <v>70000</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E19" s="11" t="n">
         <f aca="false">IF(B19="","",MAX(0,B19-$B$6))</f>
-        <v>41250</v>
+        <v>35250</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -935,14 +944,14 @@
       <c r="B20" s="13"/>
       <c r="C20" s="12"/>
       <c r="D20" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E20" s="11" t="str">
         <f aca="false">IF(B20="","",MAX(0,B20-$B$6))</f>
         <v/>
       </c>
       <c r="F20" s="12" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -952,14 +961,14 @@
       <c r="B21" s="13"/>
       <c r="C21" s="12"/>
       <c r="D21" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E21" s="11" t="str">
         <f aca="false">IF(B21="","",MAX(0,B21-$B$6))</f>
         <v/>
       </c>
       <c r="F21" s="12" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -969,14 +978,14 @@
       <c r="B22" s="13"/>
       <c r="C22" s="12"/>
       <c r="D22" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E22" s="11" t="str">
         <f aca="false">IF(B22="","",MAX(0,B22-$B$6))</f>
         <v/>
       </c>
       <c r="F22" s="12" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -986,14 +995,14 @@
       <c r="B23" s="13"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E23" s="11" t="str">
         <f aca="false">IF(B23="","",MAX(0,B23-$B$6))</f>
         <v/>
       </c>
       <c r="F23" s="12" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1003,31 +1012,35 @@
       <c r="B24" s="13"/>
       <c r="C24" s="12"/>
       <c r="D24" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E24" s="11" t="str">
         <f aca="false">IF(B24="","",MAX(0,B24-$B$6))</f>
         <v/>
       </c>
       <c r="F24" s="12" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="E25" s="11" t="str">
+      <c r="B25" s="9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E25" s="11" t="n">
         <f aca="false">IF(B25="","",MAX(0,B25-$B$6))</f>
-        <v/>
+        <v>165250</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1075,52 +1088,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>2000</v>
@@ -1148,15 +1161,15 @@
         <v>6</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C6" s="9" t="n">
         <v>2000</v>
@@ -1184,15 +1197,15 @@
         <v>6</v>
       </c>
       <c r="J6" s="12" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C7" s="9" t="n">
         <v>1500</v>
@@ -1220,15 +1233,15 @@
         <v>3</v>
       </c>
       <c r="J7" s="12" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C8" s="9" t="n">
         <v>900</v>
@@ -1256,12 +1269,12 @@
         <v>15</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E10" s="6" t="n">
         <f aca="false">SUM(E5:E8)</f>
@@ -1271,7 +1284,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E11" s="6"/>
       <c r="F11" s="6" t="n">
@@ -1281,7 +1294,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="6" t="n">

</xml_diff>

<commit_message>
Mark Astral premium milestones as skipped
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Astral_Radiance_Tracker.xlsx
+++ b/Astral_Radiance_Tracker.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="54">
   <si>
     <t xml:space="preserve">Astral Radiance Milestone Tracker</t>
   </si>
@@ -113,13 +113,10 @@
     <t xml:space="preserve">Fragments open orbs with up to 4 Astral diamonds</t>
   </si>
   <si>
-    <t xml:space="preserve">Not in screenshots yet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diamond 5 character + 400,000 gold + 100 training materials + 4,600 blue tokens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Final milestone. Out of reach with the listed tasks</t>
+    <t xml:space="preserve">Premium, requires spending money. Skipping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skipped</t>
   </si>
   <si>
     <t xml:space="preserve">How to earn points</t>
@@ -770,7 +767,7 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">MAX(0,MAX(B13:B25)-B6)</f>
-        <v>165250</v>
+        <v>35250</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -779,7 +776,7 @@
       </c>
       <c r="B11" s="6" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>27046.3804123115</v>
+        <v>5770.70484880841</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -951,7 +948,7 @@
         <v/>
       </c>
       <c r="F20" s="12" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -968,7 +965,7 @@
         <v/>
       </c>
       <c r="F21" s="12" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -985,7 +982,7 @@
         <v/>
       </c>
       <c r="F22" s="12" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1002,7 +999,7 @@
         <v/>
       </c>
       <c r="F23" s="12" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1019,28 +1016,24 @@
         <v/>
       </c>
       <c r="F24" s="12" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="B25" s="9" t="n">
-        <v>200000</v>
-      </c>
-      <c r="C25" s="10" t="s">
+      <c r="B25" s="13"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E25" s="11" t="str">
+        <f aca="false">IF(B25="","",MAX(0,B25-$B$6))</f>
+        <v/>
+      </c>
+      <c r="F25" s="12" t="s">
         <v>31</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="E25" s="11" t="n">
-        <f aca="false">IF(B25="","",MAX(0,B25-$B$6))</f>
-        <v>165250</v>
-      </c>
-      <c r="F25" s="12" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1054,7 +1047,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F13:F25" type="list">
-      <formula1>"Claimed,Not claimed"</formula1>
+      <formula1>"Claimed,Not claimed,Skipped"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1088,52 +1081,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="F4" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="J4" s="7" t="s">
         <v>43</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>45</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>46</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>2000</v>
@@ -1161,15 +1154,15 @@
         <v>6</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C6" s="9" t="n">
         <v>2000</v>
@@ -1197,15 +1190,15 @@
         <v>6</v>
       </c>
       <c r="J6" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>49</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>50</v>
       </c>
       <c r="C7" s="9" t="n">
         <v>1500</v>
@@ -1233,15 +1226,15 @@
         <v>3</v>
       </c>
       <c r="J7" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C8" s="9" t="n">
         <v>900</v>
@@ -1269,12 +1262,12 @@
         <v>15</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E10" s="6" t="n">
         <f aca="false">SUM(E5:E8)</f>
@@ -1284,7 +1277,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E11" s="6"/>
       <c r="F11" s="6" t="n">
@@ -1294,7 +1287,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="6" t="n">

</xml_diff>

<commit_message>
Add daily web store free claims to scoring
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Astral_Radiance_Tracker.xlsx
+++ b/Astral_Radiance_Tracker.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="55">
   <si>
     <t xml:space="preserve">Astral Radiance Milestone Tracker</t>
   </si>
@@ -165,6 +165,9 @@
   </si>
   <si>
     <t xml:space="preserve">Complete All Clear daily mission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Web store free claim</t>
   </si>
   <si>
     <t xml:space="preserve">Battle</t>
@@ -710,14 +713,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>34750</v>
+        <v>35500</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="6" t="n">
-        <f aca="false">B6+Scoring!F12</f>
-        <v>76750</v>
+        <f aca="false">B6+Scoring!F13</f>
+        <v>81250</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -758,7 +761,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IFERROR(INDEX(E13:E25,MATCH(TRUE(),INDEX(B13:B25&gt;B6,0),0)),0)</f>
-        <v>5250</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -767,7 +770,7 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">MAX(0,MAX(B13:B25)-B6)</f>
-        <v>35250</v>
+        <v>34500</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -776,7 +779,7 @@
       </c>
       <c r="B11" s="6" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>5770.70484880841</v>
+        <v>5775.75919096846</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -869,7 +872,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="11" t="n">
         <f aca="false">IF(B16="","",MAX(0,B16-$B$6))</f>
-        <v>5250</v>
+        <v>4500</v>
       </c>
       <c r="F16" s="12" t="s">
         <v>25</v>
@@ -888,7 +891,7 @@
       <c r="D17" s="10"/>
       <c r="E17" s="11" t="n">
         <f aca="false">IF(B17="","",MAX(0,B17-$B$6))</f>
-        <v>15250</v>
+        <v>14500</v>
       </c>
       <c r="F17" s="12" t="s">
         <v>25</v>
@@ -907,7 +910,7 @@
       <c r="D18" s="10"/>
       <c r="E18" s="11" t="n">
         <f aca="false">IF(B18="","",MAX(0,B18-$B$6))</f>
-        <v>25250</v>
+        <v>24500</v>
       </c>
       <c r="F18" s="12" t="s">
         <v>25</v>
@@ -928,7 +931,7 @@
       </c>
       <c r="E19" s="11" t="n">
         <f aca="false">IF(B19="","",MAX(0,B19-$B$6))</f>
-        <v>35250</v>
+        <v>34500</v>
       </c>
       <c r="F19" s="12" t="s">
         <v>25</v>
@@ -1066,7 +1069,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -1195,35 +1198,35 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>49</v>
-      </c>
       <c r="C7" s="9" t="n">
-        <v>1500</v>
+        <v>750</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>10500</v>
+        <v>4500</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>6000</v>
+        <v>750</v>
       </c>
       <c r="F7" s="14" t="n">
         <f aca="false">MAX(0,D7-E7)</f>
-        <v>4500</v>
+        <v>3750</v>
       </c>
       <c r="G7" s="14" t="n">
         <f aca="false">ROUNDUP(D7/C7,0)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H7" s="14" t="n">
         <f aca="false">IFERROR(INT(E7/C7),0)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I7" s="14" t="n">
         <f aca="false">IFERROR(ROUNDUP(F7/C7,0),0)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J7" s="12" t="s">
         <v>46</v>
@@ -1231,59 +1234,85 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>50</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>900</v>
+        <v>1500</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>31500</v>
+        <v>10500</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>18000</v>
+        <v>6000</v>
       </c>
       <c r="F8" s="14" t="n">
         <f aca="false">MAX(0,D8-E8)</f>
-        <v>13500</v>
+        <v>4500</v>
       </c>
       <c r="G8" s="14" t="n">
         <f aca="false">ROUNDUP(D8/C8,0)</f>
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="H8" s="14" t="n">
         <f aca="false">IFERROR(INT(E8/C8),0)</f>
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="I8" s="14" t="n">
         <f aca="false">IFERROR(ROUNDUP(F8/C8,0),0)</f>
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="J8" s="12" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="3" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E10" s="6" t="n">
-        <f aca="false">SUM(E5:E8)</f>
-        <v>28000</v>
-      </c>
-      <c r="F10" s="6"/>
+      <c r="C9" s="9" t="n">
+        <v>900</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>31500</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <f aca="false">MAX(0,D9-E9)</f>
+        <v>13500</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <f aca="false">ROUNDUP(D9/C9,0)</f>
+        <v>35</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <f aca="false">IFERROR(INT(E9/C9),0)</f>
+        <v>20</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <f aca="false">IFERROR(ROUNDUP(F9/C9,0),0)</f>
+        <v>15</v>
+      </c>
+      <c r="J9" s="12" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6" t="n">
-        <f aca="false">SUM(F5:F8)</f>
-        <v>42000</v>
-      </c>
+      <c r="E11" s="6" t="n">
+        <f aca="false">SUM(E5:E9)</f>
+        <v>28750</v>
+      </c>
+      <c r="F11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
@@ -1291,13 +1320,23 @@
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="6" t="n">
-        <f aca="false">SUMIF(J5:J8,"Yes",F5:F8)</f>
-        <v>42000</v>
+        <f aca="false">SUM(F5:F9)</f>
+        <v>45750</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6" t="n">
+        <f aca="false">SUMIF(J5:J9,"Yes",F5:F9)</f>
+        <v>45750</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J8" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J9" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Update Astral Radiance progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Astral_Radiance_Tracker.xlsx
+++ b/Astral_Radiance_Tracker.xlsx
@@ -98,10 +98,10 @@
     <t xml:space="preserve">Ancient One to 7 red stars + 200,000 gold + 25 training materials + 1,600 blue tokens</t>
   </si>
   <si>
+    <t xml:space="preserve">Emma Frost (X-Men) to 7 red stars + 250,000 gold + 30 training materials + 1,800 blue tokens</t>
+  </si>
+  <si>
     <t xml:space="preserve">Not claimed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Emma Frost (X-Men) to 7 red stars + 250,000 gold + 30 training materials + 1,800 blue tokens</t>
   </si>
   <si>
     <t xml:space="preserve">Shadow King to 7 red stars + 300,000 gold + 40 training materials + 2,400 blue tokens</t>
@@ -713,14 +713,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>35500</v>
+        <v>43500</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">B6+Scoring!F13</f>
-        <v>81250</v>
+        <v>74500</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -729,7 +729,7 @@
       </c>
       <c r="B7" s="3" t="n">
         <f aca="false">SUMPRODUCT((B13:B25&lt;&gt;"")*(B13:B25&lt;=B6))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>8</v>
@@ -745,7 +745,7 @@
       </c>
       <c r="B8" s="3" t="n">
         <f aca="false">IFERROR(INDEX(A13:A25,MATCH(TRUE(),INDEX(B13:B25&gt;B6,0),0)),"All done")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>10</v>
@@ -761,7 +761,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IFERROR(INDEX(E13:E25,MATCH(TRUE(),INDEX(B13:B25&gt;B6,0),0)),0)</f>
-        <v>4500</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -770,7 +770,7 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">MAX(0,MAX(B13:B25)-B6)</f>
-        <v>34500</v>
+        <v>26500</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -779,7 +779,7 @@
       </c>
       <c r="B11" s="6" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>5775.75919096846</v>
+        <v>4443.8995845007</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -872,10 +872,10 @@
       <c r="D16" s="10"/>
       <c r="E16" s="11" t="n">
         <f aca="false">IF(B16="","",MAX(0,B16-$B$6))</f>
-        <v>4500</v>
+        <v>0</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -886,15 +886,15 @@
         <v>50000</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="11" t="n">
         <f aca="false">IF(B17="","",MAX(0,B17-$B$6))</f>
-        <v>14500</v>
+        <v>6500</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -910,10 +910,10 @@
       <c r="D18" s="10"/>
       <c r="E18" s="11" t="n">
         <f aca="false">IF(B18="","",MAX(0,B18-$B$6))</f>
-        <v>24500</v>
+        <v>16500</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -931,10 +931,10 @@
       </c>
       <c r="E19" s="11" t="n">
         <f aca="false">IF(B19="","",MAX(0,B19-$B$6))</f>
-        <v>34500</v>
+        <v>26500</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1138,11 +1138,11 @@
         <v>14000</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="F5" s="14" t="n">
         <f aca="false">MAX(0,D5-E5)</f>
-        <v>12000</v>
+        <v>10000</v>
       </c>
       <c r="G5" s="14" t="n">
         <f aca="false">ROUNDUP(D5/C5,0)</f>
@@ -1150,11 +1150,11 @@
       </c>
       <c r="H5" s="14" t="n">
         <f aca="false">IFERROR(INT(E5/C5),0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I5" s="14" t="n">
         <f aca="false">IFERROR(ROUNDUP(F5/C5,0),0)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J5" s="12" t="s">
         <v>46</v>
@@ -1210,11 +1210,11 @@
         <v>4500</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>750</v>
+        <v>1500</v>
       </c>
       <c r="F7" s="14" t="n">
         <f aca="false">MAX(0,D7-E7)</f>
-        <v>3750</v>
+        <v>3000</v>
       </c>
       <c r="G7" s="14" t="n">
         <f aca="false">ROUNDUP(D7/C7,0)</f>
@@ -1222,11 +1222,11 @@
       </c>
       <c r="H7" s="14" t="n">
         <f aca="false">IFERROR(INT(E7/C7),0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" s="14" t="n">
         <f aca="false">IFERROR(ROUNDUP(F7/C7,0),0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J7" s="12" t="s">
         <v>46</v>
@@ -1246,11 +1246,11 @@
         <v>10500</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="F8" s="14" t="n">
         <f aca="false">MAX(0,D8-E8)</f>
-        <v>4500</v>
+        <v>1500</v>
       </c>
       <c r="G8" s="14" t="n">
         <f aca="false">ROUNDUP(D8/C8,0)</f>
@@ -1258,11 +1258,11 @@
       </c>
       <c r="H8" s="14" t="n">
         <f aca="false">IFERROR(INT(E8/C8),0)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I8" s="14" t="n">
         <f aca="false">IFERROR(ROUNDUP(F8/C8,0),0)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J8" s="12" t="s">
         <v>46</v>
@@ -1282,11 +1282,11 @@
         <v>31500</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>18000</v>
+        <v>27000</v>
       </c>
       <c r="F9" s="14" t="n">
         <f aca="false">MAX(0,D9-E9)</f>
-        <v>13500</v>
+        <v>4500</v>
       </c>
       <c r="G9" s="14" t="n">
         <f aca="false">ROUNDUP(D9/C9,0)</f>
@@ -1294,11 +1294,11 @@
       </c>
       <c r="H9" s="14" t="n">
         <f aca="false">IFERROR(INT(E9/C9),0)</f>
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I9" s="14" t="n">
         <f aca="false">IFERROR(ROUNDUP(F9/C9,0),0)</f>
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="J9" s="12" t="s">
         <v>46</v>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="E11" s="6" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>28750</v>
+        <v>43500</v>
       </c>
       <c r="F11" s="6"/>
     </row>
@@ -1321,7 +1321,7 @@
       <c r="E12" s="6"/>
       <c r="F12" s="6" t="n">
         <f aca="false">SUM(F5:F9)</f>
-        <v>45750</v>
+        <v>31000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1331,7 +1331,7 @@
       <c r="E13" s="6"/>
       <c r="F13" s="6" t="n">
         <f aca="false">SUMIF(J5:J9,"Yes",F5:F9)</f>
-        <v>45750</v>
+        <v>31000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Astral battle tasks maxed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Astral_Radiance_Tracker.xlsx
+++ b/Astral_Radiance_Tracker.xlsx
@@ -713,7 +713,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>43500</v>
+        <v>49500</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>6</v>
@@ -761,7 +761,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IFERROR(INDEX(E13:E25,MATCH(TRUE(),INDEX(B13:B25&gt;B6,0),0)),0)</f>
-        <v>6500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -770,7 +770,7 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">MAX(0,MAX(B13:B25)-B6)</f>
-        <v>26500</v>
+        <v>20500</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -779,7 +779,7 @@
       </c>
       <c r="B11" s="6" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>4443.8995845007</v>
+        <v>3550.59240567954</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -891,7 +891,7 @@
       <c r="D17" s="10"/>
       <c r="E17" s="11" t="n">
         <f aca="false">IF(B17="","",MAX(0,B17-$B$6))</f>
-        <v>6500</v>
+        <v>500</v>
       </c>
       <c r="F17" s="12" t="s">
         <v>26</v>
@@ -910,7 +910,7 @@
       <c r="D18" s="10"/>
       <c r="E18" s="11" t="n">
         <f aca="false">IF(B18="","",MAX(0,B18-$B$6))</f>
-        <v>16500</v>
+        <v>10500</v>
       </c>
       <c r="F18" s="12" t="s">
         <v>26</v>
@@ -931,7 +931,7 @@
       </c>
       <c r="E19" s="11" t="n">
         <f aca="false">IF(B19="","",MAX(0,B19-$B$6))</f>
-        <v>26500</v>
+        <v>20500</v>
       </c>
       <c r="F19" s="12" t="s">
         <v>26</v>
@@ -1246,11 +1246,11 @@
         <v>10500</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>9000</v>
+        <v>10500</v>
       </c>
       <c r="F8" s="14" t="n">
         <f aca="false">MAX(0,D8-E8)</f>
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="G8" s="14" t="n">
         <f aca="false">ROUNDUP(D8/C8,0)</f>
@@ -1258,11 +1258,11 @@
       </c>
       <c r="H8" s="14" t="n">
         <f aca="false">IFERROR(INT(E8/C8),0)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I8" s="14" t="n">
         <f aca="false">IFERROR(ROUNDUP(F8/C8,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8" s="12" t="s">
         <v>46</v>
@@ -1282,11 +1282,11 @@
         <v>31500</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>27000</v>
+        <v>31500</v>
       </c>
       <c r="F9" s="14" t="n">
         <f aca="false">MAX(0,D9-E9)</f>
-        <v>4500</v>
+        <v>0</v>
       </c>
       <c r="G9" s="14" t="n">
         <f aca="false">ROUNDUP(D9/C9,0)</f>
@@ -1294,11 +1294,11 @@
       </c>
       <c r="H9" s="14" t="n">
         <f aca="false">IFERROR(INT(E9/C9),0)</f>
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="I9" s="14" t="n">
         <f aca="false">IFERROR(ROUNDUP(F9/C9,0),0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J9" s="12" t="s">
         <v>46</v>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="E11" s="6" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>43500</v>
+        <v>49500</v>
       </c>
       <c r="F11" s="6"/>
     </row>
@@ -1321,7 +1321,7 @@
       <c r="E12" s="6"/>
       <c r="F12" s="6" t="n">
         <f aca="false">SUM(F5:F9)</f>
-        <v>31000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1331,7 +1331,7 @@
       <c r="E13" s="6"/>
       <c r="F13" s="6" t="n">
         <f aca="false">SUMIF(J5:J9,"Yes",F5:F9)</f>
-        <v>31000</v>
+        <v>25000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Morning updates: Iso-8 campaign, training store, Astral login
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Astral_Radiance_Tracker.xlsx
+++ b/Astral_Radiance_Tracker.xlsx
@@ -713,7 +713,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>49500</v>
+        <v>51500</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>6</v>
@@ -729,7 +729,7 @@
       </c>
       <c r="B7" s="3" t="n">
         <f aca="false">SUMPRODUCT((B13:B25&lt;&gt;"")*(B13:B25&lt;=B6))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>8</v>
@@ -745,14 +745,14 @@
       </c>
       <c r="B8" s="3" t="n">
         <f aca="false">IFERROR(INDEX(A13:A25,MATCH(TRUE(),INDEX(B13:B25&gt;B6,0),0)),"All done")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E8" s="3" t="n">
         <f aca="false">SUMPRODUCT((B13:B25&lt;&gt;"")*(B13:B25&lt;=B6)*(F13:F25&lt;&gt;"Claimed"))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -761,7 +761,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IFERROR(INDEX(E13:E25,MATCH(TRUE(),INDEX(B13:B25&gt;B6,0),0)),0)</f>
-        <v>500</v>
+        <v>8500</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -770,7 +770,7 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">MAX(0,MAX(B13:B25)-B6)</f>
-        <v>20500</v>
+        <v>18500</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -779,7 +779,7 @@
       </c>
       <c r="B11" s="6" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>3550.59240567954</v>
+        <v>3402.4145251131</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -891,7 +891,7 @@
       <c r="D17" s="10"/>
       <c r="E17" s="11" t="n">
         <f aca="false">IF(B17="","",MAX(0,B17-$B$6))</f>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="F17" s="12" t="s">
         <v>26</v>
@@ -910,7 +910,7 @@
       <c r="D18" s="10"/>
       <c r="E18" s="11" t="n">
         <f aca="false">IF(B18="","",MAX(0,B18-$B$6))</f>
-        <v>10500</v>
+        <v>8500</v>
       </c>
       <c r="F18" s="12" t="s">
         <v>26</v>
@@ -931,7 +931,7 @@
       </c>
       <c r="E19" s="11" t="n">
         <f aca="false">IF(B19="","",MAX(0,B19-$B$6))</f>
-        <v>20500</v>
+        <v>18500</v>
       </c>
       <c r="F19" s="12" t="s">
         <v>26</v>
@@ -1138,11 +1138,11 @@
         <v>14000</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="F5" s="14" t="n">
         <f aca="false">MAX(0,D5-E5)</f>
-        <v>10000</v>
+        <v>8000</v>
       </c>
       <c r="G5" s="14" t="n">
         <f aca="false">ROUNDUP(D5/C5,0)</f>
@@ -1150,11 +1150,11 @@
       </c>
       <c r="H5" s="14" t="n">
         <f aca="false">IFERROR(INT(E5/C5),0)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I5" s="14" t="n">
         <f aca="false">IFERROR(ROUNDUP(F5/C5,0),0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J5" s="12" t="s">
         <v>46</v>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="E11" s="6" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>49500</v>
+        <v>51500</v>
       </c>
       <c r="F11" s="6"/>
     </row>
@@ -1321,7 +1321,7 @@
       <c r="E12" s="6"/>
       <c r="F12" s="6" t="n">
         <f aca="false">SUM(F5:F9)</f>
-        <v>25000</v>
+        <v>23000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1331,7 +1331,7 @@
       <c r="E13" s="6"/>
       <c r="F13" s="6" t="n">
         <f aca="false">SUMIF(J5:J9,"Yes",F5:F9)</f>
-        <v>25000</v>
+        <v>23000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Oct 12 web store free claims, IV milestone 48
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Astral_Radiance_Tracker.xlsx
+++ b/Astral_Radiance_Tracker.xlsx
@@ -101,10 +101,10 @@
     <t xml:space="preserve">Emma Frost (X-Men) to 7 red stars + 250,000 gold + 30 training materials + 1,800 blue tokens</t>
   </si>
   <si>
+    <t xml:space="preserve">Shadow King to 7 red stars + 300,000 gold + 40 training materials + 2,400 blue tokens</t>
+  </si>
+  <si>
     <t xml:space="preserve">Not claimed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shadow King to 7 red stars + 300,000 gold + 40 training materials + 2,400 blue tokens</t>
   </si>
   <si>
     <t xml:space="preserve">1 Astral Diamond Orb fragment + 350,000 gold + 45 training materials + 2,700 blue tokens</t>
@@ -713,14 +713,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>51500</v>
+        <v>52250</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">B6+Scoring!F13</f>
-        <v>74500</v>
+        <v>75250</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -752,7 +752,7 @@
       </c>
       <c r="E8" s="3" t="n">
         <f aca="false">SUMPRODUCT((B13:B25&lt;&gt;"")*(B13:B25&lt;=B6)*(F13:F25&lt;&gt;"Claimed"))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -761,7 +761,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IFERROR(INDEX(E13:E25,MATCH(TRUE(),INDEX(B13:B25&gt;B6,0),0)),0)</f>
-        <v>8500</v>
+        <v>7750</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -770,7 +770,7 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">MAX(0,MAX(B13:B25)-B6)</f>
-        <v>18500</v>
+        <v>17750</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -779,7 +779,7 @@
       </c>
       <c r="B11" s="6" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>3402.4145251131</v>
+        <v>3573.14751200863</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -894,7 +894,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -905,15 +905,15 @@
         <v>60000</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D18" s="10"/>
       <c r="E18" s="11" t="n">
         <f aca="false">IF(B18="","",MAX(0,B18-$B$6))</f>
-        <v>8500</v>
+        <v>7750</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -931,10 +931,10 @@
       </c>
       <c r="E19" s="11" t="n">
         <f aca="false">IF(B19="","",MAX(0,B19-$B$6))</f>
-        <v>18500</v>
+        <v>17750</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Oct 14 morning: dailies, gold, Astral 61K
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B42YosRoaEhRXdGgqs1FZ4
</commit_message>
<xml_diff>
--- a/Astral_Radiance_Tracker.xlsx
+++ b/Astral_Radiance_Tracker.xlsx
@@ -104,13 +104,13 @@
     <t xml:space="preserve">Shadow King to 7 red stars + 300,000 gold + 40 training materials + 2,400 blue tokens</t>
   </si>
   <si>
+    <t xml:space="preserve">1 Astral Diamond Orb fragment + 350,000 gold + 45 training materials + 2,700 blue tokens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fragments open orbs with up to 4 Astral diamonds</t>
+  </si>
+  <si>
     <t xml:space="preserve">Not claimed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Astral Diamond Orb fragment + 350,000 gold + 45 training materials + 2,700 blue tokens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fragments open orbs with up to 4 Astral diamonds</t>
   </si>
   <si>
     <t xml:space="preserve">Premium, requires spending money. Skipping</t>
@@ -713,14 +713,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>52250</v>
+        <v>61000</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">B6+Scoring!F13</f>
-        <v>75250</v>
+        <v>84000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -729,7 +729,7 @@
       </c>
       <c r="B7" s="3" t="n">
         <f aca="false">SUMPRODUCT((B13:B25&lt;&gt;"")*(B13:B25&lt;=B6))</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>8</v>
@@ -745,7 +745,7 @@
       </c>
       <c r="B8" s="3" t="n">
         <f aca="false">IFERROR(INDEX(A13:A25,MATCH(TRUE(),INDEX(B13:B25&gt;B6,0),0)),"All done")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>10</v>
@@ -761,7 +761,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">IFERROR(INDEX(E13:E25,MATCH(TRUE(),INDEX(B13:B25&gt;B6,0),0)),0)</f>
-        <v>7750</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -770,7 +770,7 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">MAX(0,MAX(B13:B25)-B6)</f>
-        <v>17750</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -779,7 +779,7 @@
       </c>
       <c r="B11" s="6" t="n">
         <f aca="true">IFERROR(B10/MAX(B5-NOW(),0.01),0)</f>
-        <v>3573.14751200863</v>
+        <v>2610.27471574404</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -910,10 +910,10 @@
       <c r="D18" s="10"/>
       <c r="E18" s="11" t="n">
         <f aca="false">IF(B18="","",MAX(0,B18-$B$6))</f>
-        <v>7750</v>
+        <v>0</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -924,17 +924,17 @@
         <v>70000</v>
       </c>
       <c r="C19" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>28</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>29</v>
       </c>
       <c r="E19" s="11" t="n">
         <f aca="false">IF(B19="","",MAX(0,B19-$B$6))</f>
-        <v>17750</v>
+        <v>9000</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>